<commit_message>
tracking update 22.07.2026 22:31
</commit_message>
<xml_diff>
--- a/files/UAE_009_ФФЗ_22.07.2026.xlsx
+++ b/files/UAE_009_ФФЗ_22.07.2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinov\OneDrive\Desktop\РАБОЧАЯ\001 ИМПОРТ\001 containers\2026\001 UAE\UAE#9_APMG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{905DF05E-E8F9-41CB-814F-9588FFA4AAC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A47E93BC-0437-4EFA-A3AF-24A4AB553B49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -833,9 +833,9 @@
     <col min="14" max="14" width="11.5703125" style="5"/>
     <col min="15" max="15" width="11.5703125" style="7"/>
     <col min="16" max="16" width="12.5703125" style="5" customWidth="1"/>
-    <col min="17" max="17" width="18.5703125" style="5" customWidth="1"/>
-    <col min="18" max="19" width="17.5703125" style="7" customWidth="1"/>
-    <col min="20" max="20" width="14.140625" style="7" customWidth="1"/>
+    <col min="17" max="17" width="20.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="18.7109375" style="7" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="15" style="7" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="21.5703125" style="7" customWidth="1"/>
     <col min="22" max="22" width="16" style="5" customWidth="1"/>
     <col min="23" max="23" width="17.5703125" style="5" customWidth="1"/>
@@ -1999,14 +1999,14 @@
       </c>
       <c r="V2" s="62">
         <f>P2*($U$8 / $Q$6)</f>
-        <v>710.91054897045547</v>
+        <v>681.71233845207189</v>
       </c>
       <c r="W2" s="29">
         <v>810</v>
       </c>
       <c r="X2" s="63">
         <f>(W2-V2)/V2</f>
-        <v>0.13938385240315596</v>
+        <v>0.18818445011458074</v>
       </c>
       <c r="Y2" s="30">
         <f>W2*E2</f>
@@ -2014,11 +2014,11 @@
       </c>
       <c r="Z2" s="30">
         <f>E2*V2</f>
-        <v>17317780.972920295</v>
+        <v>16606512.564692471</v>
       </c>
       <c r="AA2" s="61">
         <f>V2*E2</f>
-        <v>17317780.972920295</v>
+        <v>16606512.564692471</v>
       </c>
       <c r="AB2" s="21"/>
       <c r="AC2" s="21"/>
@@ -3048,11 +3048,11 @@
       </c>
       <c r="Z3" s="58">
         <f>SUM(Z2:Z2)</f>
-        <v>17317780.972920295</v>
+        <v>16606512.564692471</v>
       </c>
       <c r="AA3" s="61">
         <f>SUM(AA2:AA2)</f>
-        <v>17317780.972920295</v>
+        <v>16606512.564692471</v>
       </c>
       <c r="AB3" s="21"/>
       <c r="AC3" s="21"/>
@@ -3206,7 +3206,7 @@
       </c>
       <c r="Z7" s="60">
         <f>(Y3-Z3)/Z3</f>
-        <v>0.13938385240315596</v>
+        <v>0.18818445011458076</v>
       </c>
     </row>
     <row r="8" spans="1:1023" ht="15.75" x14ac:dyDescent="0.25">
@@ -3227,11 +3227,11 @@
         <v>55000</v>
       </c>
       <c r="U8" s="41">
-        <v>17317780.972920295</v>
+        <v>16606512.564692469</v>
       </c>
       <c r="Z8" s="58">
         <f>Y3-Z3</f>
-        <v>2413819.0270797051</v>
+        <v>3125087.4353075288</v>
       </c>
     </row>
     <row r="9" spans="1:1023" x14ac:dyDescent="0.2">

</xml_diff>